<commit_message>
fix: resolve defaulter upload, update action API, and status display issues
</commit_message>
<xml_diff>
--- a/attendance/sample.xlsx
+++ b/attendance/sample.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\attendance3\attendance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BA6E914-A8C8-4DF1-B877-9B7B7A0C3E30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C754F67B-6A4F-4F21-8505-CA811B0E2640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="9390" windowHeight="7875" xr2:uid="{9B72A3A0-31BE-4B9F-B304-B7DC2A77795F}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="9390" windowHeight="7875" xr2:uid="{9B72A3A0-31BE-4B9F-B304-B7DC2A77795F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>Roll No</t>
   </si>
@@ -69,16 +69,28 @@
   </si>
   <si>
     <t>Dress code</t>
+  </si>
+  <si>
+    <t>24CYSE23</t>
+  </si>
+  <si>
+    <t>PRIYADHARSHINI K</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -440,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41A8ED49-4293-4739-9A53-16636F450A2E}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -483,7 +495,28 @@
         <v>10</v>
       </c>
     </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix HOD dashboard department and defaulter filtering
</commit_message>
<xml_diff>
--- a/attendance/sample.xlsx
+++ b/attendance/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\attendance3\attendance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C754F67B-6A4F-4F21-8505-CA811B0E2640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E510D5E5-3989-4BF8-9920-920E2EDF7492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2340" yWindow="2340" windowWidth="9390" windowHeight="7875" xr2:uid="{9B72A3A0-31BE-4B9F-B304-B7DC2A77795F}"/>
   </bookViews>
@@ -65,16 +65,16 @@
     <t>KAVITHA</t>
   </si>
   <si>
-    <t>CYSE</t>
-  </si>
-  <si>
     <t>Dress code</t>
   </si>
   <si>
-    <t>24CYSE23</t>
-  </si>
-  <si>
     <t>PRIYADHARSHINI K</t>
+  </si>
+  <si>
+    <t>CSE (CS)</t>
+  </si>
+  <si>
+    <t>24CYSE21</t>
   </si>
 </sst>
 </file>
@@ -489,18 +489,18 @@
         <v>2</v>
       </c>
       <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
         <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
@@ -509,10 +509,10 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
         <v>9</v>
-      </c>
-      <c r="F3" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix defaulter upload department filtering
</commit_message>
<xml_diff>
--- a/attendance/sample.xlsx
+++ b/attendance/sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Smart-Academic-System\attendance\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\attendance3\attendance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E748AE-F699-4BE7-845B-CF52C4EAF6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BD92AB-603B-4CA8-98B3-006AB6DD3660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9B72A3A0-31BE-4B9F-B304-B7DC2A77795F}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="9390" windowHeight="7875" xr2:uid="{9B72A3A0-31BE-4B9F-B304-B7DC2A77795F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -62,9 +62,6 @@
     <t>Dress code</t>
   </si>
   <si>
-    <t>CSE (CS)</t>
-  </si>
-  <si>
     <t>24CYSE01</t>
   </si>
   <si>
@@ -76,6 +73,9 @@
   </si>
   <si>
     <t>AARTHEESWARI M</t>
+  </si>
+  <si>
+    <t>CYSE (CS)</t>
   </si>
 </sst>
 </file>
@@ -457,12 +457,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41A8ED49-4293-4739-9A53-16636F450A2E}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -482,12 +482,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -496,18 +496,18 @@
         <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -516,7 +516,7 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Added assignment management and notification system
</commit_message>
<xml_diff>
--- a/attendance/sample.xlsx
+++ b/attendance/sample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\attendance3\attendance\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Smart-Academic-System\attendance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4177D8B-8F2E-40A0-9A4A-CC5404D8D22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B07E4D01-670A-43B1-AA85-B2A435640A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="9390" windowHeight="7875" xr2:uid="{9B72A3A0-31BE-4B9F-B304-B7DC2A77795F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9B72A3A0-31BE-4B9F-B304-B7DC2A77795F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -62,20 +62,20 @@
     <t>Dress code</t>
   </si>
   <si>
-    <t>24CYSE01</t>
-  </si>
-  <si>
-    <t>24CYSE02</t>
+    <t>CYSE (CS)</t>
+  </si>
+  <si>
+    <t>AASHIGA SREE L T M</t>
   </si>
   <si>
     <t xml:space="preserve">
-AAFRIN SABURA S</t>
-  </si>
-  <si>
-    <t>AARTHEESWARI M</t>
-  </si>
-  <si>
-    <t>CYSE (CS)</t>
+AISHWARYA K</t>
+  </si>
+  <si>
+    <t>24CYSE03</t>
+  </si>
+  <si>
+    <t>24CYSE04</t>
   </si>
 </sst>
 </file>
@@ -457,12 +457,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41A8ED49-4293-4739-9A53-16636F450A2E}">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -482,12 +482,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -496,18 +496,18 @@
         <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -516,7 +516,7 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F3" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Add functionality to upload defaulter list from Excel and display messages on defaulter list page
</commit_message>
<xml_diff>
--- a/attendance/sample.xlsx
+++ b/attendance/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Smart-Academic-System\attendance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B07E4D01-670A-43B1-AA85-B2A435640A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CEC43C9-61B7-4872-A11E-0BDA01F3B3B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9B72A3A0-31BE-4B9F-B304-B7DC2A77795F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Roll No</t>
   </si>
@@ -65,17 +65,10 @@
     <t>CYSE (CS)</t>
   </si>
   <si>
-    <t>AASHIGA SREE L T M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-AISHWARYA K</t>
-  </si>
-  <si>
-    <t>24CYSE03</t>
-  </si>
-  <si>
-    <t>24CYSE04</t>
+    <t>RASIKA S</t>
+  </si>
+  <si>
+    <t>24CYSE22</t>
   </si>
 </sst>
 </file>
@@ -484,7 +477,7 @@
     </row>
     <row r="2" spans="1:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>9</v>
@@ -502,25 +495,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" t="s">
-        <v>7</v>
-      </c>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B3" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Refactor HTML structure and styles in login and mentor dashboard templates; remove confirmation prompts in today leaves template
</commit_message>
<xml_diff>
--- a/attendance/sample.xlsx
+++ b/attendance/sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Smart-Academic-System\attendance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CEC43C9-61B7-4872-A11E-0BDA01F3B3B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27EB19DE-2D17-4EC8-9212-7CEFA258A46C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9B72A3A0-31BE-4B9F-B304-B7DC2A77795F}"/>
   </bookViews>
@@ -65,10 +65,11 @@
     <t>CYSE (CS)</t>
   </si>
   <si>
-    <t>RASIKA S</t>
-  </si>
-  <si>
-    <t>24CYSE22</t>
+    <t xml:space="preserve">
+AAFRIN SABURA S</t>
+  </si>
+  <si>
+    <t>24CYSE01</t>
   </si>
 </sst>
 </file>

</xml_diff>